<commit_message>
docs: hand the almanac page to Codex; update requirement statuses
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/需求记录.xlsx
+++ b/docs/需求记录.xlsx
@@ -514,10 +514,14 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>待评估</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08 提交 1e6c6d1：年/月/日/时/分下拉 + 省市区县三级联动，12 位速记保留并双向同步</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -543,10 +547,14 @@
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>待评估</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08 方案见 docs/2026-09-08-需求方案；根因 --metal 与 --earth 同色，庚辛申酉都受影响。待与老师确认要黄色的原因再定改法</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -572,10 +580,14 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>待评估</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08 提交 9d76dc8：按北京时日期判、24 项都算、每盘自动默认不覆盖手动切换</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -601,10 +613,14 @@
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>待评估</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08 数据底座已提交 6b4ab3e（1900–2100 节气冻结表，三关验证）；万年历页交 Codex，任务书 docs/2026-09-08-任务书-codex-万年历页.md</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>

<commit_message>
docs: mark REQ-004 done
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/需求记录.xlsx
+++ b/docs/需求记录.xlsx
@@ -613,12 +613,12 @@
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>进行中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08 数据底座已提交 6b4ab3e（1900–2100 节气冻结表，三关验证）；万年历页交 Codex，任务书 docs/2026-09-08-任务书-codex-万年历页.md</t>
+          <t>2026-09-08 底座 6b4ab3e + 万年历页 e853c34（Codex 实现，回执 docs/reviews/2026-09-08-回执-codex-万年历页.md）</t>
         </is>
       </c>
     </row>

</xml_diff>